<commit_message>
hig data 2025 processed
</commit_message>
<xml_diff>
--- a/data/hig/original_data/HIG_APC_2025.xlsx
+++ b/data/hig/original_data/HIG_APC_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\Forskarstöd\Open access\APC kostnader\Open APC Sweden\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4CCCDA4-666C-4C0B-837E-437E1CC12A80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F84C58A-2AF1-4772-9420-073182DEE445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A6F00635-5C01-4C60-BDF9-17EF2738987C}"/>
+    <workbookView xWindow="25620" yWindow="0" windowWidth="25980" windowHeight="20880" xr2:uid="{A6F00635-5C01-4C60-BDF9-17EF2738987C}"/>
   </bookViews>
   <sheets>
     <sheet name="HIG_APC_2025" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="48">
   <si>
     <t>institution</t>
   </si>
@@ -177,6 +177,9 @@
   </si>
   <si>
     <t>10.3390/mps8060148</t>
+  </si>
+  <si>
+    <t>10.3390/admsci15020056</t>
   </si>
 </sst>
 </file>
@@ -537,21 +540,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0416C7AE-7B3F-4B81-86CB-82046D825A9D}">
   <dimension ref="A1:K30"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.1796875" style="1"/>
-    <col min="3" max="3" width="9.1796875" style="2"/>
-    <col min="4" max="4" width="28.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.1796875" style="1"/>
-    <col min="6" max="6" width="12.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="52.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.1796875" style="1"/>
-    <col min="9" max="9" width="9.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.1796875" style="1"/>
+    <col min="1" max="2" width="9.140625" style="1"/>
+    <col min="3" max="3" width="9.140625" style="2"/>
+    <col min="4" max="4" width="28.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="1"/>
+    <col min="6" max="6" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="52.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="1"/>
+    <col min="9" max="9" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -586,7 +589,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -603,7 +606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -620,7 +623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -637,7 +640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -654,7 +657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -671,7 +674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -688,7 +691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
@@ -705,7 +708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
@@ -722,7 +725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -733,13 +736,13 @@
         <v>12964.06</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="E10" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -756,7 +759,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -773,7 +776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -790,7 +793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>11</v>
       </c>
@@ -807,7 +810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>11</v>
       </c>
@@ -824,7 +827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>11</v>
       </c>
@@ -841,7 +844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -858,7 +861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>11</v>
       </c>
@@ -875,7 +878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>11</v>
       </c>
@@ -892,7 +895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>11</v>
       </c>
@@ -909,7 +912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>11</v>
       </c>
@@ -926,7 +929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
@@ -943,7 +946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>11</v>
       </c>
@@ -960,7 +963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>11</v>
       </c>
@@ -977,7 +980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>34</v>
       </c>
@@ -1003,7 +1006,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>11</v>
       </c>
@@ -1029,7 +1032,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>11</v>
       </c>
@@ -1046,7 +1049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>11</v>
       </c>
@@ -1063,7 +1066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>11</v>
       </c>
@@ -1080,7 +1083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>11</v>
       </c>

</xml_diff>